<commit_message>
Implement compareWithFigma mobile path in BajajFinservAndroidTest
Rework BajajFinservAndroidTest into a data-driven test over Platform=
Android rows, using a SCREEN_FLOWS registry per distinct screen name
since native apps can't be navigated to generically like a web URL.
Extract BatchSupport, ComparisonResultRecorder, CompareRows,
AppiumServerSupport, and AndroidDriverFactory as shared utilities used
by both BajajFinservWebTest and BajajFinservAndroidTest, establishing
the template for future per-app comparison tests.
</commit_message>
<xml_diff>
--- a/figma-visual-testing/figma_compare_input_template.xlsx
+++ b/figma-visual-testing/figma_compare_input_template.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
@@ -433,8 +433,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
@@ -630,6 +630,53 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/abc123XYZ/My-Project?node-id=11-222</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Home Screen</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>android-home-screen</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>BajajFinservAndroidApp</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>android-home-screen-baseline</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://eyes.applitools.com/app/test-results/some-android-id</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>